<commit_message>
Modelo materiais.xlsx: sincroniza 8 materiais com posicao-estoque.xlsx
Códigos MAT-001 a MAT-008 idênticos nos dois modelos para garantir
que o catálogo exista antes da importação de estoque.

https://claude.ai/code/session_01GB592wHtRegLJEtgwh4ZdP
</commit_message>
<xml_diff>
--- a/painel/assets/modelos/materiais.xlsx
+++ b/painel/assets/modelos/materiais.xlsx
@@ -57,12 +57,10 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF777777"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -97,11 +95,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF155724"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF9C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -146,12 +139,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -519,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -539,14 +532,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preencha a partir da linha 7.</t>
+          <t>Preencha a partir da linha 7. Não altere as 6 primeiras linhas.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟢 Colunas com fundo verde são OBRIGATÓRIAS  |  Demais colunas são opcionais  |  ⚠️ Não altere as 6 primeiras linhas</t>
+          <t>🟢 Nome (col B) é OBRIGATÓRIO  |  Código é a chave única — se vazio, Nome será usado como chave  |  Decimais com vírgula</t>
         </is>
       </c>
     </row>
@@ -608,16 +601,204 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>120,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>MAT-002</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Conexão PVC 200mm</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>45,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>MAT-003</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Cimento CP-II</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>MAT-004</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Areia média</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>12,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>MAT-005</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Brita 1</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>8,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>MAT-006</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>EPI - Luvas nitrílica</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>30,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>MAT-007</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>EPI - Capacete</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>MAT-008</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Fita veda rosca</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>25,000</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A4:E4"/>
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A4:E4"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>